<commit_message>
chore: thêm log nhắc hẹn để theo dõi quá trình tạo nhắc hẹn
</commit_message>
<xml_diff>
--- a/dondathang.xlsx
+++ b/dondathang.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3120" yWindow="2310" windowWidth="23625" windowHeight="13290" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2730" yWindow="2205" windowWidth="23625" windowHeight="13290" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Don dat hang" sheetId="1" state="visible" r:id="rId1"/>
@@ -77,7 +77,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -118,6 +118,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
         <bgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -170,7 +176,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="3" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -309,6 +315,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="1" hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,19 +412,14 @@
     <author>System</author>
   </authors>
   <commentList>
+    <comment ref="Y10" authorId="0" shapeId="0">
+      <text>
+        <t>Kiểm tra lại giá mã này! - Giá hóa đơn: 146593.125 - Chênh lệch: -16287.875</t>
+      </text>
+    </comment>
     <comment ref="Y12" authorId="0" shapeId="0">
       <text>
-        <t>Kiểm tra lại giá mã này! - Giá hóa đơn: 162272.0 - Chênh lệch: 32454.399999999994</t>
-      </text>
-    </comment>
-    <comment ref="Y13" authorId="0" shapeId="0">
-      <text>
-        <t>Kiểm tra lại giá mã này! - Giá hóa đơn: 71014.0 - Chênh lệch: 14202.800000000003</t>
-      </text>
-    </comment>
-    <comment ref="Y20" authorId="0" shapeId="0">
-      <text>
-        <t>Kiểm tra lại giá mã này! - Giá hóa đơn: 59114.0 - Chênh lệch: 11822.800000000003</t>
+        <t>Kiểm tra lại giá mã này! - Giá hóa đơn: 146593.125 - Chênh lệch: -16287.875</t>
       </text>
     </comment>
   </commentList>
@@ -749,7 +751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV20"/>
+  <dimension ref="A1:AV13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.7109375" customWidth="1" style="30" min="1" max="1"/>
@@ -803,8 +805,8 @@
     <col width="9.140625" customWidth="1" style="14" min="49" max="50"/>
     <col width="31.42578125" customWidth="1" style="14" min="51" max="51"/>
     <col width="13.7109375" customWidth="1" style="14" min="52" max="52"/>
-    <col width="9.140625" customWidth="1" style="14" min="53" max="1108"/>
-    <col width="9.140625" customWidth="1" style="14" min="1109" max="16384"/>
+    <col width="9.140625" customWidth="1" style="14" min="53" max="1109"/>
+    <col width="9.140625" customWidth="1" style="14" min="1110" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="20.25" customHeight="1" s="45">
@@ -819,7 +821,7 @@
       <c r="E1" s="32" t="n"/>
       <c r="F1" s="32" t="n"/>
       <c r="G1" s="40" t="n">
-        <v>4069</v>
+        <v>4084</v>
       </c>
       <c r="H1" s="6" t="n"/>
       <c r="I1" s="33" t="n"/>
@@ -1373,7 +1375,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ĐĐHWINMART-4192677025</t>
+          <t>ĐĐHCOOP-102592451-00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1383,27 +1385,27 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>16/07/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1354-WMP_AMBIENT_CAN THO_FT - 1354 - WMP_AMBIENT_CAN THO_FT Đường 3A, Khu Công Nghiệp Sông Hậu – Giai Đoạn 1, Xã Châu Thành, TP. Cần Thơ TP. Cần Thơ Việt Nam</t>
+          <t>09167-CF HN YEN NGHIA - B9 - Lô B- TT2, dự án khu nhà ở Bộ tư lệnh Thủ Đô, phường Yên Nghĩa, Thành phố Hà Nội</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MN_MT_WIN1352</t>
+          <t>MB_MT_CF9167</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>WINMART PO4192677025 - Nguyễn Trọng Tùng (Admin)_0855004420_tungnt4@sup (Tổng trọng lượng: 13.9 kg)</t>
+          <t>COOPFOOD PO102592451-00 (Tổng trọng lượng: 182.4 kg)</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t xml:space="preserve">WINMART PO4192677025 </t>
+          <t>COOPFOOD PO102592451-00</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1418,7 +1420,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>LA_KHO2026</t>
+          <t>TP_HN_12</t>
         </is>
       </c>
       <c r="X9" t="n">
@@ -1435,12 +1437,12 @@
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>MT_MN</t>
+          <t>MT_MB</t>
         </is>
       </c>
       <c r="AM9" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>HN</t>
         </is>
       </c>
       <c r="AV9" t="n">
@@ -1455,7 +1457,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ĐĐHWINMART-4192677025</t>
+          <t>ĐĐHCOOP-102592451-00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1465,32 +1467,32 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16/07/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1354-WMP_AMBIENT_CAN THO_FT - 1354 - WMP_AMBIENT_CAN THO_FT Đường 3A, Khu Công Nghiệp Sông Hậu – Giai Đoạn 1, Xã Châu Thành, TP. Cần Thơ TP. Cần Thơ Việt Nam</t>
+          <t>09167-CF HN YEN NGHIA - B9 - Lô B- TT2, dự án khu nhà ở Bộ tư lệnh Thủ Đô, phường Yên Nghĩa, Thành phố Hà Nội</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>MN_MT_WIN1352</t>
+          <t>MB_MT_CF9167</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>WINMART PO4192677025 - Nguyễn Trọng Tùng (Admin)_0855004420_tungnt4@sup</t>
+          <t>COOPFOOD PO102592451-00</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>TP31630</t>
+          <t>TP30879_02</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Nước rửa chén Blue hương Chanh túi 3.2L (QC*4)</t>
+          <t>Nước giặt xả Blue Đậm đặc Hương Thảo Mộc túi 3.6L</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1505,14 +1507,14 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>LA_KHO2026</t>
+          <t>TP_HN_12</t>
         </is>
       </c>
       <c r="X10" t="n">
-        <v>4</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>56811.2</v>
+        <v>12</v>
+      </c>
+      <c r="Y10" s="49" t="n">
+        <v>162881</v>
       </c>
       <c r="Z10">
         <f>Y10*X10</f>
@@ -1523,24 +1525,34 @@
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>MT_MN</t>
+          <t>MT_MB</t>
         </is>
       </c>
       <c r="AM10" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>HN</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>KM Bó Kèm - Che Barcode</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>0879_0879_1</t>
         </is>
       </c>
       <c r="AQ10" t="inlineStr">
         <is>
-          <t>Giảm 20%</t>
+          <t>1+1</t>
         </is>
       </c>
       <c r="AT10" t="n">
-        <v>13.9</v>
+        <v>45.6</v>
       </c>
       <c r="AU10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AV10" t="n">
         <v>60</v>
@@ -1549,12 +1561,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>09/07/2026</t>
+          <t>08/07/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ĐĐHWINMART-4901304749</t>
+          <t>ĐĐHCOOP-102592451-00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1564,46 +1576,51 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>17/07/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1325-WMP_AMBIENT_DA NANG_FT - 1325 - WMP_AMBIENT_DA NANG_FT Đường số 6 KCN Hòa Khánh TP. Đà Nẵng Việt Nam</t>
+          <t>09167-CF HN YEN NGHIA - B9 - Lô B- TT2, dự án khu nhà ở Bộ tư lệnh Thủ Đô, phường Yên Nghĩa, Thành phố Hà Nội</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>MN_MT_WIN1326</t>
+          <t>MB_MT_CF9167</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>WINMART PO4901304749 (Tổng trọng lượng: 580.3 kg)</t>
+          <t>COOPFOOD PO102592451-00</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>TP30879_02</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>WINMART PO4901304749</t>
+          <t>Nước giặt xả Blue Đậm đặc Hương Thảo Mộc túi 3.6L</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>TP_DN_1</t>
+          <t>TP_HN_12</t>
         </is>
       </c>
       <c r="X11" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="Y11" t="n">
         <v>0</v>
@@ -1616,13 +1633,24 @@
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>MT_MN</t>
+          <t>MT_MB</t>
         </is>
       </c>
       <c r="AM11" t="inlineStr">
         <is>
-          <t>DN</t>
-        </is>
+          <t>HN</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>0879_0879_1</t>
+        </is>
+      </c>
+      <c r="AT11" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>3</v>
       </c>
       <c r="AV11" t="n">
         <v>60</v>
@@ -1631,12 +1659,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>09/07/2026</t>
+          <t>08/07/2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ĐĐHWINMART-4901304749</t>
+          <t>ĐĐHCOOP-102592451-00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1646,32 +1674,32 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>17/07/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1325-WMP_AMBIENT_DA NANG_FT - 1325 - WMP_AMBIENT_DA NANG_FT Đường số 6 KCN Hòa Khánh TP. Đà Nẵng Việt Nam</t>
+          <t>09167-CF HN YEN NGHIA - B9 - Lô B- TT2, dự án khu nhà ở Bộ tư lệnh Thủ Đô, phường Yên Nghĩa, Thành phố Hà Nội</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>MN_MT_WIN1326</t>
+          <t>MB_MT_CF9167</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>WINMART PO4901304749</t>
+          <t>COOPFOOD PO102592451-00</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>TP31203</t>
+          <t>TP30886_02</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Nước Giặt Blue kháng khuẩn hương hoa thạch thảo 3.2L</t>
+          <t>Nước giặt xả Blue Đậm đặc Hương Nước Hoa túi 3.6L</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1686,14 +1714,14 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>TP_DN_1</t>
+          <t>TP_HN_12</t>
         </is>
       </c>
       <c r="X12" t="n">
-        <v>8</v>
-      </c>
-      <c r="Y12" s="46" t="n">
-        <v>162272</v>
+        <v>12</v>
+      </c>
+      <c r="Y12" s="49" t="n">
+        <v>162881</v>
       </c>
       <c r="Z12">
         <f>Y12*X12</f>
@@ -1704,24 +1732,34 @@
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>MT_MN</t>
+          <t>MT_MB</t>
         </is>
       </c>
       <c r="AM12" t="inlineStr">
         <is>
-          <t>DN</t>
+          <t>HN</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>KM Bó Kèm - Che Barcode</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>0886_0886_1</t>
         </is>
       </c>
       <c r="AQ12" t="inlineStr">
         <is>
-          <t>Giảm 20%</t>
+          <t>1+1</t>
         </is>
       </c>
       <c r="AT12" t="n">
-        <v>27.8</v>
+        <v>45.6</v>
       </c>
       <c r="AU12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AV12" t="n">
         <v>60</v>
@@ -1730,12 +1768,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>09/07/2026</t>
+          <t>08/07/2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ĐĐHWINMART-4901304749</t>
+          <t>ĐĐHCOOP-102592451-00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1745,32 +1783,32 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>17/07/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1325-WMP_AMBIENT_DA NANG_FT - 1325 - WMP_AMBIENT_DA NANG_FT Đường số 6 KCN Hòa Khánh TP. Đà Nẵng Việt Nam</t>
+          <t>09167-CF HN YEN NGHIA - B9 - Lô B- TT2, dự án khu nhà ở Bộ tư lệnh Thủ Đô, phường Yên Nghĩa, Thành phố Hà Nội</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>MN_MT_WIN1326</t>
+          <t>MB_MT_CF9167</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>WINMART PO4901304749</t>
+          <t>COOPFOOD PO102592451-00</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>TP31630</t>
+          <t>TP30886_02</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Nước rửa chén Blue hương Chanh túi 3.2L (QC*4)</t>
+          <t>Nước giặt xả Blue Đậm đặc Hương Nước Hoa túi 3.6L</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1780,760 +1818,48 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Không</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>TP_DN_1</t>
+          <t>TP_HN_12</t>
         </is>
       </c>
       <c r="X13" t="n">
         <v>12</v>
       </c>
-      <c r="Y13" s="46" t="n">
-        <v>71014</v>
-      </c>
-      <c r="Z13">
-        <f>Y13*X13</f>
-        <v/>
+      <c r="Y13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0</v>
       </c>
       <c r="AE13" t="n">
         <v>8</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>MT_MN</t>
+          <t>MT_MB</t>
         </is>
       </c>
       <c r="AM13" t="inlineStr">
         <is>
-          <t>DN</t>
-        </is>
-      </c>
-      <c r="AQ13" t="inlineStr">
-        <is>
-          <t>Giảm 20%</t>
+          <t>HN</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>0886_0886_1</t>
         </is>
       </c>
       <c r="AT13" t="n">
-        <v>41.7</v>
+        <v>45.6</v>
       </c>
       <c r="AU13" t="n">
         <v>3</v>
       </c>
       <c r="AV13" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>ĐĐHWINMART-4901304749</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Chưa thực hiện</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>17/07/2026</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>1325-WMP_AMBIENT_DA NANG_FT - 1325 - WMP_AMBIENT_DA NANG_FT Đường số 6 KCN Hòa Khánh TP. Đà Nẵng Việt Nam</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>MN_MT_WIN1326</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>WINMART PO4901304749</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>TP32767</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>Nước lau sàn Blue Hương Lavender túi 3.5kg</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>TP_DN_1</t>
-        </is>
-      </c>
-      <c r="X14" t="n">
-        <v>8</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>71600</v>
-      </c>
-      <c r="Z14">
-        <f>Y14*X14</f>
-        <v/>
-      </c>
-      <c r="AE14" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ14" t="inlineStr">
-        <is>
-          <t>MT_MN</t>
-        </is>
-      </c>
-      <c r="AM14" t="inlineStr">
-        <is>
-          <t>DN</t>
-        </is>
-      </c>
-      <c r="AO14" t="inlineStr">
-        <is>
-          <t>KM Giao Rời - Không Che</t>
-        </is>
-      </c>
-      <c r="AQ14" t="inlineStr">
-        <is>
-          <t>1+1 {KM Giao Rời - Không che barcode}</t>
-        </is>
-      </c>
-      <c r="AT14" t="n">
-        <v>28.8</v>
-      </c>
-      <c r="AU14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AV14" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>ĐĐHWINMART-4901304749</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Chưa thực hiện</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>17/07/2026</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>1325-WMP_AMBIENT_DA NANG_FT - 1325 - WMP_AMBIENT_DA NANG_FT Đường số 6 KCN Hòa Khánh TP. Đà Nẵng Việt Nam</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>MN_MT_WIN1326</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>WINMART PO4901304749</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>TP32767</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>Nước lau sàn Blue Hương Lavender túi 3.5kg</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>TP_DN_1</t>
-        </is>
-      </c>
-      <c r="X15" t="n">
-        <v>8</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE15" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ15" t="inlineStr">
-        <is>
-          <t>MT_MN</t>
-        </is>
-      </c>
-      <c r="AM15" t="inlineStr">
-        <is>
-          <t>DN</t>
-        </is>
-      </c>
-      <c r="AT15" t="n">
-        <v>28.8</v>
-      </c>
-      <c r="AU15" t="n">
-        <v>2</v>
-      </c>
-      <c r="AV15" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>ĐĐHWINMART-4901304749</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Chưa thực hiện</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>17/07/2026</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>1325-WMP_AMBIENT_DA NANG_FT - 1325 - WMP_AMBIENT_DA NANG_FT Đường số 6 KCN Hòa Khánh TP. Đà Nẵng Việt Nam</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>MN_MT_WIN1326</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>WINMART PO4901304749</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>TP30879_02</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>Nước giặt xả Blue Đậm đặc Hương Thảo Mộc túi 3.6L</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>TP_DN_1</t>
-        </is>
-      </c>
-      <c r="X16" t="n">
-        <v>32</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>145000</v>
-      </c>
-      <c r="Z16">
-        <f>Y16*X16</f>
-        <v/>
-      </c>
-      <c r="AE16" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ16" t="inlineStr">
-        <is>
-          <t>MT_MN</t>
-        </is>
-      </c>
-      <c r="AM16" t="inlineStr">
-        <is>
-          <t>DN</t>
-        </is>
-      </c>
-      <c r="AO16" t="inlineStr">
-        <is>
-          <t>KM Bó Kèm + Che barcode</t>
-        </is>
-      </c>
-      <c r="AP16" t="inlineStr">
-        <is>
-          <t>0879_0879_1</t>
-        </is>
-      </c>
-      <c r="AQ16" t="inlineStr">
-        <is>
-          <t>1+1  {KM Bó Kèm + Che barcode}</t>
-        </is>
-      </c>
-      <c r="AT16" t="n">
-        <v>121.6</v>
-      </c>
-      <c r="AU16" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV16" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>ĐĐHWINMART-4901304749</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Chưa thực hiện</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>17/07/2026</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>1325-WMP_AMBIENT_DA NANG_FT - 1325 - WMP_AMBIENT_DA NANG_FT Đường số 6 KCN Hòa Khánh TP. Đà Nẵng Việt Nam</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>MN_MT_WIN1326</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>WINMART PO4901304749</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>TP30879_02</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>Nước giặt xả Blue Đậm đặc Hương Thảo Mộc túi 3.6L</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>TP_DN_1</t>
-        </is>
-      </c>
-      <c r="X17" t="n">
-        <v>32</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE17" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ17" t="inlineStr">
-        <is>
-          <t>MT_MN</t>
-        </is>
-      </c>
-      <c r="AM17" t="inlineStr">
-        <is>
-          <t>DN</t>
-        </is>
-      </c>
-      <c r="AP17" t="inlineStr">
-        <is>
-          <t>0879_0879_1</t>
-        </is>
-      </c>
-      <c r="AT17" t="n">
-        <v>121.6</v>
-      </c>
-      <c r="AU17" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV17" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>ĐĐHWINMART-4901304749</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Chưa thực hiện</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>17/07/2026</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>1325-WMP_AMBIENT_DA NANG_FT - 1325 - WMP_AMBIENT_DA NANG_FT Đường số 6 KCN Hòa Khánh TP. Đà Nẵng Việt Nam</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>MN_MT_WIN1326</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>WINMART PO4901304749</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>TP30886_02</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>Nước giặt xả Blue Đậm đặc Hương Nước Hoa túi 3.6L</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>TP_DN_1</t>
-        </is>
-      </c>
-      <c r="X18" t="n">
-        <v>24</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>145000</v>
-      </c>
-      <c r="Z18">
-        <f>Y18*X18</f>
-        <v/>
-      </c>
-      <c r="AE18" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ18" t="inlineStr">
-        <is>
-          <t>MT_MN</t>
-        </is>
-      </c>
-      <c r="AM18" t="inlineStr">
-        <is>
-          <t>DN</t>
-        </is>
-      </c>
-      <c r="AO18" t="inlineStr">
-        <is>
-          <t>KM Bó Kèm + Che barcode</t>
-        </is>
-      </c>
-      <c r="AP18" t="inlineStr">
-        <is>
-          <t>0886_0886_1</t>
-        </is>
-      </c>
-      <c r="AQ18" t="inlineStr">
-        <is>
-          <t>1+1  {KM Bó Kèm + Che barcode}</t>
-        </is>
-      </c>
-      <c r="AT18" t="n">
-        <v>91.2</v>
-      </c>
-      <c r="AU18" t="n">
-        <v>6</v>
-      </c>
-      <c r="AV18" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>ĐĐHWINMART-4901304749</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Chưa thực hiện</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>17/07/2026</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>1325-WMP_AMBIENT_DA NANG_FT - 1325 - WMP_AMBIENT_DA NANG_FT Đường số 6 KCN Hòa Khánh TP. Đà Nẵng Việt Nam</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>MN_MT_WIN1326</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>WINMART PO4901304749</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>TP30886_02</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>Nước giặt xả Blue Đậm đặc Hương Nước Hoa túi 3.6L</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>TP_DN_1</t>
-        </is>
-      </c>
-      <c r="X19" t="n">
-        <v>24</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE19" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ19" t="inlineStr">
-        <is>
-          <t>MT_MN</t>
-        </is>
-      </c>
-      <c r="AM19" t="inlineStr">
-        <is>
-          <t>DN</t>
-        </is>
-      </c>
-      <c r="AP19" t="inlineStr">
-        <is>
-          <t>0886_0886_1</t>
-        </is>
-      </c>
-      <c r="AT19" t="n">
-        <v>91.2</v>
-      </c>
-      <c r="AU19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AV19" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>ĐĐHWINMART-4901304749</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Chưa thực hiện</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>17/07/2026</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>1325-WMP_AMBIENT_DA NANG_FT - 1325 - WMP_AMBIENT_DA NANG_FT Đường số 6 KCN Hòa Khánh TP. Đà Nẵng Việt Nam</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>MN_MT_WIN1326</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>WINMART PO4901304749</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>TP30473</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>Nước rửa chén Blue chiết xuất gạo túi 2.1L (QC*6)</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>TP_DN_1</t>
-        </is>
-      </c>
-      <c r="X20" t="n">
-        <v>12</v>
-      </c>
-      <c r="Y20" s="46" t="n">
-        <v>59114</v>
-      </c>
-      <c r="Z20">
-        <f>Y20*X20</f>
-        <v/>
-      </c>
-      <c r="AE20" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ20" t="inlineStr">
-        <is>
-          <t>MT_MN</t>
-        </is>
-      </c>
-      <c r="AM20" t="inlineStr">
-        <is>
-          <t>DN</t>
-        </is>
-      </c>
-      <c r="AQ20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Giảm 20%
-</t>
-        </is>
-      </c>
-      <c r="AT20" t="n">
-        <v>27.6</v>
-      </c>
-      <c r="AU20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AV20" t="n">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: cập nhật file Excel "n hằng tay"
</commit_message>
<xml_diff>
--- a/dondathang.xlsx
+++ b/dondathang.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2730" yWindow="2205" windowWidth="23625" windowHeight="13290" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Don dat hang" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Don dat hang" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="SAVoucher">#REF!</definedName>
@@ -404,26 +404,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>System</author>
-  </authors>
-  <commentList>
-    <comment ref="Y10" authorId="0" shapeId="0">
-      <text>
-        <t>Kiểm tra lại giá mã này! - Giá hóa đơn: 146593.125 - Chênh lệch: -16287.875</t>
-      </text>
-    </comment>
-    <comment ref="Y12" authorId="0" shapeId="0">
-      <text>
-        <t>Kiểm tra lại giá mã này! - Giá hóa đơn: 146593.125 - Chênh lệch: -16287.875</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -751,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV13"/>
+  <dimension ref="A1:AV11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.7109375" customWidth="1" style="30" min="1" max="1"/>
@@ -821,7 +801,7 @@
       <c r="E1" s="32" t="n"/>
       <c r="F1" s="32" t="n"/>
       <c r="G1" s="40" t="n">
-        <v>4084</v>
+        <v>4114</v>
       </c>
       <c r="H1" s="6" t="n"/>
       <c r="I1" s="33" t="n"/>
@@ -1370,12 +1350,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>08/07/2026</t>
+          <t>09/07/2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ĐĐHCOOP-102592451-00</t>
+          <t>ĐĐHSATRA-P-005484027</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1385,27 +1365,27 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>11/07/2026</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>09167-CF HN YEN NGHIA - B9 - Lô B- TT2, dự án khu nhà ở Bộ tư lệnh Thủ Đô, phường Yên Nghĩa, Thành phố Hà Nội</t>
+          <t>3/1 Nguyễn Thị Định, Phường Bình Trưng,HCM,VNM</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MB_MT_CF9167</t>
+          <t>MN_MT_STF1150</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>COOPFOOD PO102592451-00 (Tổng trọng lượng: 182.4 kg)</t>
+          <t>SATRA P-005484027  (Tổng trọng lượng: 30.4 kg)</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>COOPFOOD PO102592451-00</t>
+          <t>SATRA P-005484027</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1420,7 +1400,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>TP_HN_12</t>
+          <t>LA_TP</t>
         </is>
       </c>
       <c r="X9" t="n">
@@ -1437,12 +1417,12 @@
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>MT_MB</t>
+          <t>MT_MN</t>
         </is>
       </c>
       <c r="AM9" t="inlineStr">
         <is>
-          <t>HN</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="AV9" t="n">
@@ -1452,12 +1432,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>08/07/2026</t>
+          <t>09/07/2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ĐĐHCOOP-102592451-00</t>
+          <t>ĐĐHSATRA-P-005484027</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1467,32 +1447,32 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>11/07/2026</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>09167-CF HN YEN NGHIA - B9 - Lô B- TT2, dự án khu nhà ở Bộ tư lệnh Thủ Đô, phường Yên Nghĩa, Thành phố Hà Nội</t>
+          <t>3/1 Nguyễn Thị Định, Phường Bình Trưng,HCM,VNM</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>MB_MT_CF9167</t>
+          <t>MN_MT_STF1150</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>COOPFOOD PO102592451-00</t>
+          <t xml:space="preserve">SATRA P-005484027 </t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>TP30879_02</t>
+          <t>TP30985_02</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Nước giặt xả Blue Đậm đặc Hương Thảo Mộc túi 3.6L</t>
+          <t>Nước giặt xả Blue Deep Clean Hương Thanh Xuân Túi 3.6L</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1507,14 +1487,14 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>TP_HN_12</t>
+          <t>LA_TP</t>
         </is>
       </c>
       <c r="X10" t="n">
-        <v>12</v>
-      </c>
-      <c r="Y10" s="49" t="n">
-        <v>162881</v>
+        <v>4</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>107100</v>
       </c>
       <c r="Z10">
         <f>Y10*X10</f>
@@ -1525,34 +1505,24 @@
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>MT_MB</t>
+          <t>MT_MN</t>
         </is>
       </c>
       <c r="AM10" t="inlineStr">
         <is>
-          <t>HN</t>
-        </is>
-      </c>
-      <c r="AO10" t="inlineStr">
-        <is>
-          <t>KM Bó Kèm - Che Barcode</t>
-        </is>
-      </c>
-      <c r="AP10" t="inlineStr">
-        <is>
-          <t>0879_0879_1</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="AQ10" t="inlineStr">
         <is>
-          <t>1+1</t>
+          <t>Giảm 40%</t>
         </is>
       </c>
       <c r="AT10" t="n">
-        <v>45.6</v>
+        <v>15.2</v>
       </c>
       <c r="AU10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AV10" t="n">
         <v>60</v>
@@ -1561,12 +1531,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08/07/2026</t>
+          <t>09/07/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ĐĐHCOOP-102592451-00</t>
+          <t>ĐĐHSATRA-P-005484027</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1576,32 +1546,32 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>11/07/2026</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>09167-CF HN YEN NGHIA - B9 - Lô B- TT2, dự án khu nhà ở Bộ tư lệnh Thủ Đô, phường Yên Nghĩa, Thành phố Hà Nội</t>
+          <t>3/1 Nguyễn Thị Định, Phường Bình Trưng,HCM,VNM</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>MB_MT_CF9167</t>
+          <t>MN_MT_STF1150</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>COOPFOOD PO102592451-00</t>
+          <t xml:space="preserve">SATRA P-005484027 </t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>TP30879_02</t>
+          <t>TP30992_02</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Nước giặt xả Blue Đậm đặc Hương Thảo Mộc túi 3.6L</t>
+          <t>Nước giặt xả Blue Deep Clean Hương Phấn Hồng Túi 3.6L</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1611,255 +1581,49 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Không</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>TP_HN_12</t>
+          <t>LA_TP</t>
         </is>
       </c>
       <c r="X11" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="Y11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>0</v>
+        <v>107100</v>
+      </c>
+      <c r="Z11">
+        <f>Y11*X11</f>
+        <v/>
       </c>
       <c r="AE11" t="n">
         <v>8</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>MT_MB</t>
+          <t>MT_MN</t>
         </is>
       </c>
       <c r="AM11" t="inlineStr">
         <is>
-          <t>HN</t>
-        </is>
-      </c>
-      <c r="AP11" t="inlineStr">
-        <is>
-          <t>0879_0879_1</t>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>Giảm 40%</t>
         </is>
       </c>
       <c r="AT11" t="n">
-        <v>45.6</v>
+        <v>15.2</v>
       </c>
       <c r="AU11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AV11" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>ĐĐHCOOP-102592451-00</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Chưa thực hiện</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>09167-CF HN YEN NGHIA - B9 - Lô B- TT2, dự án khu nhà ở Bộ tư lệnh Thủ Đô, phường Yên Nghĩa, Thành phố Hà Nội</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>MB_MT_CF9167</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>COOPFOOD PO102592451-00</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>TP30886_02</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>Nước giặt xả Blue Đậm đặc Hương Nước Hoa túi 3.6L</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>TP_HN_12</t>
-        </is>
-      </c>
-      <c r="X12" t="n">
-        <v>12</v>
-      </c>
-      <c r="Y12" s="49" t="n">
-        <v>162881</v>
-      </c>
-      <c r="Z12">
-        <f>Y12*X12</f>
-        <v/>
-      </c>
-      <c r="AE12" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ12" t="inlineStr">
-        <is>
-          <t>MT_MB</t>
-        </is>
-      </c>
-      <c r="AM12" t="inlineStr">
-        <is>
-          <t>HN</t>
-        </is>
-      </c>
-      <c r="AO12" t="inlineStr">
-        <is>
-          <t>KM Bó Kèm - Che Barcode</t>
-        </is>
-      </c>
-      <c r="AP12" t="inlineStr">
-        <is>
-          <t>0886_0886_1</t>
-        </is>
-      </c>
-      <c r="AQ12" t="inlineStr">
-        <is>
-          <t>1+1</t>
-        </is>
-      </c>
-      <c r="AT12" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="AU12" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV12" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>ĐĐHCOOP-102592451-00</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Chưa thực hiện</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>09167-CF HN YEN NGHIA - B9 - Lô B- TT2, dự án khu nhà ở Bộ tư lệnh Thủ Đô, phường Yên Nghĩa, Thành phố Hà Nội</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>MB_MT_CF9167</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>COOPFOOD PO102592451-00</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>TP30886_02</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>Nước giặt xả Blue Đậm đặc Hương Nước Hoa túi 3.6L</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>TP_HN_12</t>
-        </is>
-      </c>
-      <c r="X13" t="n">
-        <v>12</v>
-      </c>
-      <c r="Y13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE13" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ13" t="inlineStr">
-        <is>
-          <t>MT_MB</t>
-        </is>
-      </c>
-      <c r="AM13" t="inlineStr">
-        <is>
-          <t>HN</t>
-        </is>
-      </c>
-      <c r="AP13" t="inlineStr">
-        <is>
-          <t>0886_0886_1</t>
-        </is>
-      </c>
-      <c r="AT13" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="AU13" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV13" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1917,7 +1681,6 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>